<commit_message>
Llegadas del 31/10/2026: 5 reservas anotadas en Ingresos Diarios y reporte
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NwDrgkMJkDdMQQno5kfhvB
</commit_message>
<xml_diff>
--- a/reportes/reservas_2026-10-31.xlsx
+++ b/reportes/reservas_2026-10-31.xlsx
@@ -60,9 +60,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -430,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -474,17 +475,157 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2bdr Condo 6</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Jonathan Solano Alvarado</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>293.2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>3bdr Villa in Uvita TOUCAN</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Francisco Salazar barboza</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Booking.com</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>197.32</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>4bdr House in Uvita LORO</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Verónica Blanco Fernández</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>283.54</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4bdr House in Uvita QUETZAL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Yeiner Gonzalez</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>191.65</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Love Nest in Uvita</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Luis Diego Rojas</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>303.9999999999999</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="F2" s="3" t="n">
-        <v>0</v>
+      <c r="F7" s="4" t="n">
+        <v>1269.71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>